<commit_message>
test(factory): add support for multiple test data scenarios
</commit_message>
<xml_diff>
--- a/BlazeDemo/src/test/resources/testdata/FlightBookingData.xlsx
+++ b/BlazeDemo/src/test/resources/testdata/FlightBookingData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\git\Wipro-SDET\BlazeDemo\src\test\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\git\Wipro-Capstone-Project\BlazeDemo\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C485F3-3977-4345-BB6E-E82E1D83D338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D822C974-17BD-4699-95A2-6AB443A43EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
   <si>
     <t>CardNumber</t>
   </si>
@@ -69,7 +69,55 @@
     <t>Park Street Area</t>
   </si>
   <si>
-    <t>Baivab Sarakr</t>
+    <t>DepartureCity</t>
+  </si>
+  <si>
+    <t>DestinationCity</t>
+  </si>
+  <si>
+    <t>Boston</t>
+  </si>
+  <si>
+    <t>London</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>Rome</t>
+  </si>
+  <si>
+    <t>American Express</t>
+  </si>
+  <si>
+    <t>Mexico City</t>
+  </si>
+  <si>
+    <t>Dublin</t>
+  </si>
+  <si>
+    <t>Baivab Sarkar</t>
+  </si>
+  <si>
+    <t>Ayush Sharma</t>
+  </si>
+  <si>
+    <t>Harsh Choudhary</t>
+  </si>
+  <si>
+    <t>Park Circus</t>
+  </si>
+  <si>
+    <t>College Street</t>
+  </si>
+  <si>
+    <t>Howrah</t>
+  </si>
+  <si>
+    <t>DumDum</t>
+  </si>
+  <si>
+    <t>Diner's Club</t>
   </si>
 </sst>
 </file>
@@ -113,16 +161,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,78 +489,174 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="9.140625" style="2"/>
-    <col min="7" max="7" width="18" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5703125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="F2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="1">
+      <c r="G2" s="3">
         <v>700001</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="H2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="4">
+        <v>4111111111111110</v>
+      </c>
+      <c r="J2" s="3">
         <v>12</v>
       </c>
-      <c r="G2" s="3">
-        <v>4111111111111110</v>
-      </c>
-      <c r="H2" s="1">
+      <c r="K2" s="3">
+        <v>2028</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="3">
+        <v>745501</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="1">
-        <v>2028</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>14</v>
+      <c r="I3" s="4">
+        <v>378282246310005</v>
+      </c>
+      <c r="J3" s="3">
+        <v>10</v>
+      </c>
+      <c r="K3" s="3">
+        <v>2029</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="3">
+        <v>798457</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I4" s="4">
+        <v>30569309025904</v>
+      </c>
+      <c r="J4" s="3">
+        <v>9</v>
+      </c>
+      <c r="K4" s="3">
+        <v>2030</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>